<commit_message>
feat: update customer import template generation and validation; enhance import process with new column structure and placeholder email handling
</commit_message>
<xml_diff>
--- a/public/templates/customer-import-template.xlsx
+++ b/public/templates/customer-import-template.xlsx
@@ -398,161 +398,197 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:M2"/>
   <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="40.83203125" customWidth="1"/>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="34.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="32.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>email</v>
+        <v>ID</v>
       </c>
       <c r="B1" t="str">
-        <v>first_name</v>
+        <v>Full-name</v>
       </c>
       <c r="C1" t="str">
-        <v>last_name</v>
+        <v>StreetAddress</v>
       </c>
       <c r="D1" t="str">
-        <v>phone</v>
+        <v>Locality</v>
       </c>
       <c r="E1" t="str">
-        <v>address</v>
+        <v>Postcode</v>
+      </c>
+      <c r="F1" t="str">
+        <v>State</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Region</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Phone-Fixed</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Phone-Mobile</v>
+      </c>
+      <c r="J1" t="str">
+        <v>DNCR-Phone-Fixed</v>
+      </c>
+      <c r="K1" t="str">
+        <v>DNCR-Mobile</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Email</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Status</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>jane.smith@example.com</v>
+        <v>4414754</v>
       </c>
       <c r="B2" t="str">
-        <v>Jane</v>
+        <v>Alex Stolbnyak</v>
       </c>
       <c r="C2" t="str">
-        <v>Smith</v>
+        <v>19 Urlovskya Street</v>
       </c>
       <c r="D2" t="str">
-        <v>0412 345 678</v>
+        <v>SYDNEY</v>
       </c>
       <c r="E2" t="str">
-        <v>12 Solar St, Sydney NSW 2000</v>
+        <v>1001</v>
+      </c>
+      <c r="F2" t="str">
+        <v>NSW</v>
+      </c>
+      <c r="G2" t="str">
+        <v>SYDNEY</v>
+      </c>
+      <c r="H2" t="str">
+        <v>0636285153</v>
+      </c>
+      <c r="I2" t="str">
+        <v>0412345678</v>
+      </c>
+      <c r="J2" t="str">
+        <v>N</v>
+      </c>
+      <c r="K2" t="str">
+        <v>N</v>
+      </c>
+      <c r="L2" t="str">
+        <v>alex.stolbnyak@example.com</v>
+      </c>
+      <c r="M2" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A15"/>
   <cols>
-    <col min="1" max="1" width="88.83203125" customWidth="1"/>
+    <col min="1" max="1" width="92.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Customer import template</v>
+        <v/>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>Columns</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>1. Fill one row per customer on the Customers sheet.</v>
+        <v xml:space="preserve">  • ID — Your source system's ID. Used to match on re-import.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2. Do not rename or reorder the header row (email, first_name, last_name, phone, address).</v>
+        <v xml:space="preserve">  • Full-name (required) — Full name. First word is the given name, the rest the surname.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>3. Required columns: email, first_name, last_name.</v>
+        <v xml:space="preserve">  • StreetAddress — Street number and name</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>4. Optional columns: phone, address.</v>
+        <v xml:space="preserve">  • Locality — Suburb or town</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v/>
+        <v xml:space="preserve">  • Postcode — Postcode</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Email</v>
+        <v xml:space="preserve">  • State — State, e.g. NSW</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v xml:space="preserve">  • Must be a valid address and unique in the platform.</v>
+        <v xml:space="preserve">  • Region — Region. Ignored when it repeats Locality.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v xml:space="preserve">  • Duplicate emails in your file or already registered are skipped on import.</v>
+        <v xml:space="preserve">  • Phone-Fixed — Landline</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v/>
+        <v xml:space="preserve">  • Phone-Mobile — Mobile. Preferred over the landline when both are present.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Phone (Australia)</v>
+        <v xml:space="preserve">  • DNCR-Phone-Fixed — Landline on the Do Not Call Register? Y/N</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v xml:space="preserve">  • Examples: 0412 345 678, +61 412 345 678, (02) 9123 4567</v>
+        <v xml:space="preserve">  • DNCR-Mobile — Mobile on the Do Not Call Register? Y/N</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v xml:space="preserve">  • Leave blank if unknown.</v>
+        <v xml:space="preserve">  • Email — Leave blank if unknown — a placeholder is generated.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Google Sheets</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v xml:space="preserve">  • File → Download → Microsoft Excel (.xlsx) or Comma-separated values (.csv), then upload in the installer portal.</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>Delete the sample row before importing your real customers.</v>
+        <v xml:space="preserve">  • Status — Free-text status from your source system</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>